<commit_message>
Update: kurs fix, daily prices, WP articles 2026-06-29
</commit_message>
<xml_diff>
--- a/data/bi_rate_inflasi.xlsx
+++ b/data/bi_rate_inflasi.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,18 +455,42 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>5.77</v>
       </c>
       <c r="C2" t="n">
-        <v>0.18</v>
+        <v>0.38</v>
       </c>
       <c r="D2" t="n">
-        <v>2.34</v>
+        <v>2.13</v>
       </c>
       <c r="E2" t="n">
-        <v>108.48</v>
+        <v>108.4</v>
       </c>
       <c r="F2" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="E3" t="n">
+        <v>108.51</v>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>fallback (last known)</t>
         </is>

</xml_diff>

<commit_message>
fix: BBM silent when no confirmed changes
</commit_message>
<xml_diff>
--- a/data/bi_rate_inflasi.xlsx
+++ b/data/bi_rate_inflasi.xlsx
@@ -479,16 +479,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6.08</v>
+        <v>6.17</v>
       </c>
       <c r="C3" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="D3" t="n">
-        <v>2.05</v>
+        <v>2.19</v>
       </c>
       <c r="E3" t="n">
-        <v>108.51</v>
+        <v>108.37</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: tambah script update_pakan_nutrisi.py + kurs/bbm fix
</commit_message>
<xml_diff>
--- a/data/bi_rate_inflasi.xlsx
+++ b/data/bi_rate_inflasi.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,18 +479,42 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6.17</v>
+        <v>6.27</v>
       </c>
       <c r="C3" t="n">
-        <v>0.58</v>
+        <v>0.63</v>
       </c>
       <c r="D3" t="n">
-        <v>2.19</v>
+        <v>2.16</v>
       </c>
       <c r="E3" t="n">
-        <v>108.37</v>
+        <v>108.17</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="E4" t="n">
+        <v>108.26</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>fallback (last known)</t>
         </is>

</xml_diff>

<commit_message>
fix: dedup Excel, backfill historis 30 hari (minyak/BiRate/CPO/pertanian/kurs)
</commit_message>
<xml_diff>
--- a/data/bi_rate_inflasi.xlsx
+++ b/data/bi_rate_inflasi.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -503,21 +503,591 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6.2</v>
+        <v>5.89</v>
       </c>
       <c r="C4" t="n">
-        <v>0.62</v>
+        <v>0.73</v>
       </c>
       <c r="D4" t="n">
-        <v>2.29</v>
+        <v>2.4</v>
       </c>
       <c r="E4" t="n">
-        <v>108.26</v>
+        <v>108.12</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>fallback (last known)</t>
         </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="E5" t="n">
+        <v>146.4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="E6" t="n">
+        <v>146.11</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>145.24</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="E8" t="n">
+        <v>146.39</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.84</v>
+      </c>
+      <c r="E9" t="n">
+        <v>144.96</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>6</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="E10" t="n">
+        <v>144.91</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="E11" t="n">
+        <v>144.58</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>6</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="E12" t="n">
+        <v>145.12</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>6</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="E13" t="n">
+        <v>144.98</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>6</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="E14" t="n">
+        <v>145.26</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>6</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="E15" t="n">
+        <v>145.73</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>6</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="E16" t="n">
+        <v>144.61</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="D17" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="E17" t="n">
+        <v>145.58</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>6</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="E18" t="n">
+        <v>144.99</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D19" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="E19" t="n">
+        <v>146.49</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>6</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="E20" t="n">
+        <v>144.83</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>6</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="E21" t="n">
+        <v>145.67</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>6</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="D22" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="E22" t="n">
+        <v>145.74</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>6</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="D23" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="E23" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>6</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="D24" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="E24" t="n">
+        <v>145.73</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>6</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="D25" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="E25" t="n">
+        <v>145.36</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>6</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D26" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="E26" t="n">
+        <v>146.19</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>6</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="D27" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="E27" t="n">
+        <v>145.85</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>6</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="D28" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="E28" t="n">
+        <v>146.2</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>6</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D29" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="E29" t="n">
+        <v>144.73</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>6</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="D30" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="E30" t="n">
+        <v>146.33</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>6</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="D31" t="n">
+        <v>2.84</v>
+      </c>
+      <c r="E31" t="n">
+        <v>144.55</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D32" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="E32" t="n">
+        <v>146.28</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>6</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="D33" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="E33" t="n">
+        <v>145.41</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>6</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="D34" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="E34" t="n">
+        <v>145.43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: crypto/emas data path + recovery loader from JSON history
</commit_message>
<xml_diff>
--- a/data/bi_rate_inflasi.xlsx
+++ b/data/bi_rate_inflasi.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1090,6 +1090,30 @@
         <v>145.43</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D35" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E35" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: 3 bugs - crypto 429 retry + import paths + master_update sys.path
</commit_message>
<xml_diff>
--- a/data/bi_rate_inflasi.xlsx
+++ b/data/bi_rate_inflasi.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Harian" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Harian" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
fix: dedup harga_sembako 221→35 rows, fix dedup key (was referencing missing column)
</commit_message>
<xml_diff>
--- a/data/bi_rate_inflasi.xlsx
+++ b/data/bi_rate_inflasi.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Harian" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Harian" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1114,6 +1114,54 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D36" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E36" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D37" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E37" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: dedup pertanian_ternak 111→38 + auto_dedup 1715 rows across 19 files
</commit_message>
<xml_diff>
--- a/data/bi_rate_inflasi.xlsx
+++ b/data/bi_rate_inflasi.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Harian" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Harian" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1162,6 +1162,30 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D38" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E38" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: sembako card - show items with actual data (beras prem/med, gas elpiji)
</commit_message>
<xml_diff>
--- a/data/bi_rate_inflasi.xlsx
+++ b/data/bi_rate_inflasi.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Harian" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Harian" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1186,6 +1186,30 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D39" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E39" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: excel data corrupt rows + wp article data-driven
</commit_message>
<xml_diff>
--- a/data/bi_rate_inflasi.xlsx
+++ b/data/bi_rate_inflasi.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1210,6 +1210,54 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D40" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E40" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D41" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E41" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: 3 bugs - add_row 24-col mapping, crypto IDR from OHLC, wp article data-driven
</commit_message>
<xml_diff>
--- a/data/bi_rate_inflasi.xlsx
+++ b/data/bi_rate_inflasi.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Harian" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Harian" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1258,6 +1258,30 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D42" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E42" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: crypto 31s (3 coins, less sleep) + watchdog <1s
</commit_message>
<xml_diff>
--- a/data/bi_rate_inflasi.xlsx
+++ b/data/bi_rate_inflasi.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1306,6 +1306,30 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D44" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E44" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: copy latest crypto fix to scripts
</commit_message>
<xml_diff>
--- a/data/bi_rate_inflasi.xlsx
+++ b/data/bi_rate_inflasi.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1330,6 +1330,78 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D45" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E45" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D46" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E46" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D47" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E47" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(charts): all 6 chart cards wrapped in chart-wrapper(320px/280px), chart-grid replaces chart-row, rm min-height:100vh & flex:1 causing tall cards
</commit_message>
<xml_diff>
--- a/data/bi_rate_inflasi.xlsx
+++ b/data/bi_rate_inflasi.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1402,6 +1402,54 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D48" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E48" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D49" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E49" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
backup: AI analysis system + data updates
- core/ai/ — full AI analysis pipeline (providers, agents, job runner, store)
- app.py — AI analysis endpoints + rate limiter fix
- Data updates: crypto, emas, saham, sembako, sentimen
- Web UI updates (script.js, index.html)
- Script updates (create_excel, update_crypto, update_harga)
</commit_message>
<xml_diff>
--- a/data/bi_rate_inflasi.xlsx
+++ b/data/bi_rate_inflasi.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1450,6 +1450,198 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D50" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E50" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C51" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D51" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E51" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D52" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E52" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C53" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D53" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E53" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C54" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D54" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E54" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C55" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D55" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E55" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C56" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D56" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E56" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="C57" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D57" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E57" t="n">
+        <v>108.12</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>fallback (last known)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>